<commit_message>
Add gabay_name field + display_name property; update all templates
- User.gabay_name: nickname used in leads/reports/Lazada (Karen, Arvie, etc.)
- User.display_name: property returning gabay_name or full_name fallback
- /admin/migrate-gabay-name: adds column + populates 9 agents
- All report/lead templates now use display_name instead of full_name
- Admin user forms still show full_name

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LAZADAleads.xlsx
+++ b/LAZADAleads.xlsx
@@ -15460,6 +15460,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:O905"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="64.42578125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="61" t="s">
@@ -52952,12 +52955,12 @@
   </sheetData>
   <autoFilter ref="A2:O2"/>
   <mergeCells count="6">
+    <mergeCell ref="H1:O1"/>
     <mergeCell ref="E884:E885"/>
     <mergeCell ref="F884:F885"/>
     <mergeCell ref="E886:E888"/>
     <mergeCell ref="F886:F888"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="H1:O1"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="G3" r:id="rId1"/>

</xml_diff>